<commit_message>
Fix P&L formulas not displaying and rename revenue category
Inject cached formula values into the P&L sheet's XML so the numbers
render immediately in any viewer (LibreOffice can't run in this
sandbox to do a normal recalc, and openpyxl-written formulas have no
cached value until something computes them). Also rename "Membership
Fee" to "SEO & Web Services" to match the Patriot Software category
name for the $99/mo charge.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EWHJ4JSrXozykE2fwAhg1g
</commit_message>
<xml_diff>
--- a/Practice Budget Expenses Revenue Conversion/2026 P&L by Month.xlsx
+++ b/Practice Budget Expenses Revenue Conversion/2026 P&L by Month.xlsx
@@ -584,48 +584,48 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Membership Fee ($99/mo)</t>
+          <t>SEO &amp; Web Services ($99/mo)</t>
         </is>
       </c>
       <c r="B6" s="9">
-        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"Membership Fee",'Revenue Detail'!$A:$A,"&gt;="&amp;B$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
-        <v/>
+        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"SEO &amp; Web Services",'Revenue Detail'!$A:$A,"&gt;="&amp;B$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
+        <v>198</v>
       </c>
       <c r="C6" s="9">
-        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"Membership Fee",'Revenue Detail'!$A:$A,"&gt;="&amp;C$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
-        <v/>
+        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"SEO &amp; Web Services",'Revenue Detail'!$A:$A,"&gt;="&amp;C$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
+        <v>0</v>
       </c>
       <c r="D6" s="9">
-        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"Membership Fee",'Revenue Detail'!$A:$A,"&gt;="&amp;D$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
-        <v/>
+        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"SEO &amp; Web Services",'Revenue Detail'!$A:$A,"&gt;="&amp;D$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
+        <v>396</v>
       </c>
       <c r="E6" s="9">
-        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"Membership Fee",'Revenue Detail'!$A:$A,"&gt;="&amp;E$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
-        <v/>
+        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"SEO &amp; Web Services",'Revenue Detail'!$A:$A,"&gt;="&amp;E$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
+        <v>0</v>
       </c>
       <c r="F6" s="9">
-        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"Membership Fee",'Revenue Detail'!$A:$A,"&gt;="&amp;F$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
-        <v/>
+        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"SEO &amp; Web Services",'Revenue Detail'!$A:$A,"&gt;="&amp;F$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
+        <v>198</v>
       </c>
       <c r="G6" s="9">
-        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"Membership Fee",'Revenue Detail'!$A:$A,"&gt;="&amp;G$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
-        <v/>
+        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"SEO &amp; Web Services",'Revenue Detail'!$A:$A,"&gt;="&amp;G$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
+        <v>198</v>
       </c>
       <c r="H6" s="9">
-        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"Membership Fee",'Revenue Detail'!$A:$A,"&gt;="&amp;H$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
-        <v/>
+        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"SEO &amp; Web Services",'Revenue Detail'!$A:$A,"&gt;="&amp;H$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
+        <v>198</v>
       </c>
       <c r="I6" s="9">
-        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"Membership Fee",'Revenue Detail'!$A:$A,"&gt;="&amp;I$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
-        <v/>
+        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"SEO &amp; Web Services",'Revenue Detail'!$A:$A,"&gt;="&amp;I$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
+        <v>297</v>
       </c>
       <c r="J6" s="9">
-        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"Membership Fee",'Revenue Detail'!$A:$A,"&gt;="&amp;J$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
-        <v/>
+        <f>SUMIFS('Revenue Detail'!$D:$D,'Revenue Detail'!$C:$C,"SEO &amp; Web Services",'Revenue Detail'!$A:$A,"&gt;="&amp;J$4,'Revenue Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
+        <v>0</v>
       </c>
       <c r="K6" s="9">
         <f>SUM(B6:J6)</f>
-        <v/>
+        <v>1485</v>
       </c>
     </row>
     <row r="7">
@@ -636,43 +636,43 @@
       </c>
       <c r="B7" s="10">
         <f>SUM(B6:B6)</f>
-        <v/>
+        <v>198</v>
       </c>
       <c r="C7" s="10">
         <f>SUM(C6:C6)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="D7" s="10">
         <f>SUM(D6:D6)</f>
-        <v/>
+        <v>396</v>
       </c>
       <c r="E7" s="10">
         <f>SUM(E6:E6)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F7" s="10">
         <f>SUM(F6:F6)</f>
-        <v/>
+        <v>198</v>
       </c>
       <c r="G7" s="10">
         <f>SUM(G6:G6)</f>
-        <v/>
+        <v>198</v>
       </c>
       <c r="H7" s="10">
         <f>SUM(H6:H6)</f>
-        <v/>
+        <v>198</v>
       </c>
       <c r="I7" s="10">
         <f>SUM(I6:I6)</f>
-        <v/>
+        <v>297</v>
       </c>
       <c r="J7" s="10">
         <f>SUM(J6:J6)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K7" s="10">
         <f>SUM(K6:K6)</f>
-        <v/>
+        <v>1485</v>
       </c>
     </row>
     <row r="9">
@@ -700,43 +700,43 @@
       </c>
       <c r="B10" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;B$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
-        <v/>
+        <v>20</v>
       </c>
       <c r="C10" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;C$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
-        <v/>
+        <v>20</v>
       </c>
       <c r="D10" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;D$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
-        <v/>
+        <v>20</v>
       </c>
       <c r="E10" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;E$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
-        <v/>
+        <v>20</v>
       </c>
       <c r="F10" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;F$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
-        <v/>
+        <v>20</v>
       </c>
       <c r="G10" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;G$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
-        <v/>
+        <v>20</v>
       </c>
       <c r="H10" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;H$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
-        <v/>
+        <v>20</v>
       </c>
       <c r="I10" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;I$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
-        <v/>
+        <v>20</v>
       </c>
       <c r="J10" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;J$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
-        <v/>
+        <v>30</v>
       </c>
       <c r="K10" s="9">
         <f>SUM(B10:J10)</f>
-        <v/>
+        <v>190</v>
       </c>
     </row>
     <row r="11">
@@ -747,43 +747,43 @@
       </c>
       <c r="B11" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;B$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="C11" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;C$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="D11" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;D$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="E11" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;E$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="F11" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;F$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="G11" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;G$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="H11" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;H$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="I11" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;I$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="J11" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;J$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
-        <v/>
+        <v>10</v>
       </c>
       <c r="K11" s="9">
         <f>SUM(B11:J11)</f>
-        <v/>
+        <v>90</v>
       </c>
     </row>
     <row r="12">
@@ -794,43 +794,43 @@
       </c>
       <c r="B12" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;B$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="C12" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;C$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="D12" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;D$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="E12" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;E$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="F12" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;F$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="G12" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;G$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="H12" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;H$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="I12" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;I$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="J12" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;J$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
-        <v/>
+        <v>12</v>
       </c>
       <c r="K12" s="9">
         <f>SUM(B12:J12)</f>
-        <v/>
+        <v>108</v>
       </c>
     </row>
     <row r="13">
@@ -841,43 +841,43 @@
       </c>
       <c r="B13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;B$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="C13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;C$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="D13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;D$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="E13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;E$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="F13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;F$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="G13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;G$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="H13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;H$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="I13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;I$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="J13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;J$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
-        <v/>
+        <v>9</v>
       </c>
       <c r="K13" s="9">
         <f>SUM(B13:J13)</f>
-        <v/>
+        <v>57</v>
       </c>
     </row>
     <row r="14">
@@ -888,43 +888,43 @@
       </c>
       <c r="B14" s="10">
         <f>SUM(B10:B13)</f>
-        <v/>
+        <v>48</v>
       </c>
       <c r="C14" s="10">
         <f>SUM(C10:C13)</f>
-        <v/>
+        <v>48</v>
       </c>
       <c r="D14" s="10">
         <f>SUM(D10:D13)</f>
-        <v/>
+        <v>48</v>
       </c>
       <c r="E14" s="10">
         <f>SUM(E10:E13)</f>
-        <v/>
+        <v>48</v>
       </c>
       <c r="F14" s="10">
         <f>SUM(F10:F13)</f>
-        <v/>
+        <v>48</v>
       </c>
       <c r="G14" s="10">
         <f>SUM(G10:G13)</f>
-        <v/>
+        <v>48</v>
       </c>
       <c r="H14" s="10">
         <f>SUM(H10:H13)</f>
-        <v/>
+        <v>48</v>
       </c>
       <c r="I14" s="10">
         <f>SUM(I10:I13)</f>
-        <v/>
+        <v>48</v>
       </c>
       <c r="J14" s="10">
         <f>SUM(J10:J13)</f>
-        <v/>
+        <v>61</v>
       </c>
       <c r="K14" s="10">
         <f>SUM(K10:K13)</f>
-        <v/>
+        <v>445</v>
       </c>
     </row>
     <row r="16">
@@ -935,43 +935,43 @@
       </c>
       <c r="B16" s="12">
         <f>B7-B14</f>
-        <v/>
+        <v>150</v>
       </c>
       <c r="C16" s="12">
         <f>C7-C14</f>
-        <v/>
+        <v>-48</v>
       </c>
       <c r="D16" s="12">
         <f>D7-D14</f>
-        <v/>
+        <v>348</v>
       </c>
       <c r="E16" s="12">
         <f>E7-E14</f>
-        <v/>
+        <v>-48</v>
       </c>
       <c r="F16" s="12">
         <f>F7-F14</f>
-        <v/>
+        <v>150</v>
       </c>
       <c r="G16" s="12">
         <f>G7-G14</f>
-        <v/>
+        <v>150</v>
       </c>
       <c r="H16" s="12">
         <f>H7-H14</f>
-        <v/>
+        <v>150</v>
       </c>
       <c r="I16" s="12">
         <f>I7-I14</f>
-        <v/>
+        <v>249</v>
       </c>
       <c r="J16" s="12">
         <f>J7-J14</f>
-        <v/>
+        <v>-61</v>
       </c>
       <c r="K16" s="12">
         <f>K7-K14</f>
-        <v/>
+        <v>1040</v>
       </c>
     </row>
     <row r="19">
@@ -984,14 +984,14 @@
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>- Membership Fee revenue is pulled directly from the recorded Invoice rows in Revenue-source.xlsx (actual invoice dates, not evenly smoothed).</t>
+          <t>- SEO &amp; Web Services revenue is pulled directly from the recorded Invoice rows in Revenue-source.xlsx (actual invoice dates, not evenly smoothed).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Feb and Apr show $0 because no invoice was recorded those months in the source file; Sep shows $0 because no Sep membership invoice has been recorded yet.</t>
+          <t xml:space="preserve">  Feb and Apr show $0 because no invoice was recorded those months in the source file; Sep shows $0 because no Sep SEO &amp; Web Services invoice has been recorded yet.</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>Membership Fee</t>
+          <t>SEO &amp; Web Services</t>
         </is>
       </c>
       <c r="D2" s="17" t="n">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Membership Fee</t>
+          <t>SEO &amp; Web Services</t>
         </is>
       </c>
       <c r="D3" s="17" t="n">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Membership Fee</t>
+          <t>SEO &amp; Web Services</t>
         </is>
       </c>
       <c r="D4" s="17" t="n">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Membership Fee</t>
+          <t>SEO &amp; Web Services</t>
         </is>
       </c>
       <c r="D5" s="17" t="n">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Membership Fee</t>
+          <t>SEO &amp; Web Services</t>
         </is>
       </c>
       <c r="D6" s="17" t="n">
@@ -1173,7 +1173,7 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Membership Fee</t>
+          <t>SEO &amp; Web Services</t>
         </is>
       </c>
       <c r="D7" s="17" t="n">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Membership Fee</t>
+          <t>SEO &amp; Web Services</t>
         </is>
       </c>
       <c r="D8" s="17" t="n">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Membership Fee</t>
+          <t>SEO &amp; Web Services</t>
         </is>
       </c>
       <c r="D9" s="17" t="n">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Membership Fee</t>
+          <t>SEO &amp; Web Services</t>
         </is>
       </c>
       <c r="D10" s="17" t="n">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Membership Fee</t>
+          <t>SEO &amp; Web Services</t>
         </is>
       </c>
       <c r="D11" s="17" t="n">
@@ -1263,7 +1263,7 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Membership Fee</t>
+          <t>SEO &amp; Web Services</t>
         </is>
       </c>
       <c r="D12" s="17" t="n">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Membership Fee</t>
+          <t>SEO &amp; Web Services</t>
         </is>
       </c>
       <c r="D13" s="17" t="n">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Membership Fee</t>
+          <t>SEO &amp; Web Services</t>
         </is>
       </c>
       <c r="D14" s="17" t="n">
@@ -1317,7 +1317,7 @@
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Membership Fee</t>
+          <t>SEO &amp; Web Services</t>
         </is>
       </c>
       <c r="D15" s="17" t="n">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Membership Fee</t>
+          <t>SEO &amp; Web Services</t>
         </is>
       </c>
       <c r="D16" s="17" t="n">

</xml_diff>

<commit_message>
Restructure P&L with COGS / Gross Profit / Operating Expenses
Split Hosting and SEO Tools (Seobility + Ubersuggest) out as COGS
since they're direct per-client costs of delivering SEO & Web
Services; keep the $3/mo QuickBooks Payments processing fee (renamed
Bank Fees) as an Operating Expense below Gross Profit. Add a GL
Account reference column to Expense Detail mapping each cost to its
Patriot account (GroupRB:Hosting, GroupRB:SEO Tools,
GroupRB:Bank Fees).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EWHJ4JSrXozykE2fwAhg1g
</commit_message>
<xml_diff>
--- a/Practice Budget Expenses Revenue Conversion/2026 P&L by Month.xlsx
+++ b/Practice Budget Expenses Revenue Conversion/2026 P&L by Month.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="166" formatCode="$#,##0;($#,##0);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,11 @@
     <font>
       <name val="Arial"/>
       <color rgb="00000000"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="006B7280"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -110,30 +115,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="17" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -499,10 +506,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
@@ -678,7 +685,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Expenses</t>
+          <t>Cost of Goods Sold (COGS)</t>
         </is>
       </c>
       <c r="B9" s="7" t="n"/>
@@ -695,336 +702,515 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t xml:space="preserve">    Seobility</t>
         </is>
       </c>
       <c r="B10" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;B$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
+        <v>10</v>
+      </c>
+      <c r="C10" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;C$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
+        <v>10</v>
+      </c>
+      <c r="D10" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;D$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
+        <v>10</v>
+      </c>
+      <c r="E10" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;E$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
+        <v>10</v>
+      </c>
+      <c r="F10" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;F$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
+        <v>10</v>
+      </c>
+      <c r="G10" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;G$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
+        <v>10</v>
+      </c>
+      <c r="H10" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;H$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
+        <v>10</v>
+      </c>
+      <c r="I10" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;I$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
+        <v>10</v>
+      </c>
+      <c r="J10" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;J$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
+        <v>10</v>
+      </c>
+      <c r="K10" s="9">
+        <f>SUM(B10:J10)</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    Ubersuggest</t>
+        </is>
+      </c>
+      <c r="B11" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;B$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
+        <v>12</v>
+      </c>
+      <c r="C11" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;C$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
+        <v>12</v>
+      </c>
+      <c r="D11" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;D$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
+        <v>12</v>
+      </c>
+      <c r="E11" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;E$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
+        <v>12</v>
+      </c>
+      <c r="F11" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;F$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
+        <v>12</v>
+      </c>
+      <c r="G11" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;G$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
+        <v>12</v>
+      </c>
+      <c r="H11" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;H$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
+        <v>12</v>
+      </c>
+      <c r="I11" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;I$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
+        <v>12</v>
+      </c>
+      <c r="J11" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;J$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
+        <v>12</v>
+      </c>
+      <c r="K11" s="9">
+        <f>SUM(B11:J11)</f>
+        <v>108</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>SEO Tools (GroupRB:SEO Tools)</t>
+        </is>
+      </c>
+      <c r="B12" s="9">
+        <f>SUM(B10:B11)</f>
+        <v>22</v>
+      </c>
+      <c r="C12" s="9">
+        <f>SUM(C10:C11)</f>
+        <v>22</v>
+      </c>
+      <c r="D12" s="9">
+        <f>SUM(D10:D11)</f>
+        <v>22</v>
+      </c>
+      <c r="E12" s="9">
+        <f>SUM(E10:E11)</f>
+        <v>22</v>
+      </c>
+      <c r="F12" s="9">
+        <f>SUM(F10:F11)</f>
+        <v>22</v>
+      </c>
+      <c r="G12" s="9">
+        <f>SUM(G10:G11)</f>
+        <v>22</v>
+      </c>
+      <c r="H12" s="9">
+        <f>SUM(H10:H11)</f>
+        <v>22</v>
+      </c>
+      <c r="I12" s="9">
+        <f>SUM(I10:I11)</f>
+        <v>22</v>
+      </c>
+      <c r="J12" s="9">
+        <f>SUM(J10:J11)</f>
+        <v>22</v>
+      </c>
+      <c r="K12" s="9">
+        <f>SUM(K10:K11)</f>
+        <v>198</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Hosting (GroupRB:Hosting)</t>
+        </is>
+      </c>
+      <c r="B13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;B$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
         <v>20</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;C$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
         <v>20</v>
       </c>
-      <c r="D10" s="9">
+      <c r="D13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;D$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
         <v>20</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;E$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
         <v>20</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;F$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
         <v>20</v>
       </c>
-      <c r="G10" s="9">
+      <c r="G13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;G$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
         <v>20</v>
       </c>
-      <c r="H10" s="9">
+      <c r="H13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;H$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
         <v>20</v>
       </c>
-      <c r="I10" s="9">
+      <c r="I13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;I$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
         <v>20</v>
       </c>
-      <c r="J10" s="9">
+      <c r="J13" s="9">
         <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;J$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
         <v>30</v>
       </c>
-      <c r="K10" s="9">
-        <f>SUM(B10:J10)</f>
-        <v>190</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>Seobility</t>
-        </is>
-      </c>
-      <c r="B11" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;B$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
-        <v>10</v>
-      </c>
-      <c r="C11" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;C$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
-        <v>10</v>
-      </c>
-      <c r="D11" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;D$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
-        <v>10</v>
-      </c>
-      <c r="E11" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;E$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
-        <v>10</v>
-      </c>
-      <c r="F11" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;F$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
-        <v>10</v>
-      </c>
-      <c r="G11" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;G$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
-        <v>10</v>
-      </c>
-      <c r="H11" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;H$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
-        <v>10</v>
-      </c>
-      <c r="I11" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;I$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
-        <v>10</v>
-      </c>
-      <c r="J11" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Seobility",'Expense Detail'!$A:$A,"&gt;="&amp;J$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
-        <v>10</v>
-      </c>
-      <c r="K11" s="9">
-        <f>SUM(B11:J11)</f>
-        <v>90</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>Ubersuggest</t>
-        </is>
-      </c>
-      <c r="B12" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;B$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
-        <v>12</v>
-      </c>
-      <c r="C12" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;C$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
-        <v>12</v>
-      </c>
-      <c r="D12" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;D$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
-        <v>12</v>
-      </c>
-      <c r="E12" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;E$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
-        <v>12</v>
-      </c>
-      <c r="F12" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;F$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
-        <v>12</v>
-      </c>
-      <c r="G12" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;G$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
-        <v>12</v>
-      </c>
-      <c r="H12" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;H$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
-        <v>12</v>
-      </c>
-      <c r="I12" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;I$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
-        <v>12</v>
-      </c>
-      <c r="J12" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Ubersuggest",'Expense Detail'!$A:$A,"&gt;="&amp;J$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
-        <v>12</v>
-      </c>
-      <c r="K12" s="9">
-        <f>SUM(B12:J12)</f>
-        <v>108</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="B13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;B$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
-        <v>6</v>
-      </c>
-      <c r="C13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;C$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
-        <v>6</v>
-      </c>
-      <c r="D13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;D$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
-        <v>6</v>
-      </c>
-      <c r="E13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;E$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
-        <v>6</v>
-      </c>
-      <c r="F13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;F$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
-        <v>6</v>
-      </c>
-      <c r="G13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;G$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
-        <v>6</v>
-      </c>
-      <c r="H13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;H$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
-        <v>6</v>
-      </c>
-      <c r="I13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;I$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
-        <v>6</v>
-      </c>
-      <c r="J13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Billing Fee",'Expense Detail'!$A:$A,"&gt;="&amp;J$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
-        <v>9</v>
-      </c>
       <c r="K13" s="9">
         <f>SUM(B13:J13)</f>
-        <v>57</v>
+        <v>190</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Total Expenses</t>
+          <t>Total COGS</t>
         </is>
       </c>
       <c r="B14" s="10">
-        <f>SUM(B10:B13)</f>
-        <v>48</v>
+        <f>SUM(B12:B13)</f>
+        <v>42</v>
       </c>
       <c r="C14" s="10">
-        <f>SUM(C10:C13)</f>
-        <v>48</v>
+        <f>SUM(C12:C13)</f>
+        <v>42</v>
       </c>
       <c r="D14" s="10">
-        <f>SUM(D10:D13)</f>
-        <v>48</v>
+        <f>SUM(D12:D13)</f>
+        <v>42</v>
       </c>
       <c r="E14" s="10">
-        <f>SUM(E10:E13)</f>
-        <v>48</v>
+        <f>SUM(E12:E13)</f>
+        <v>42</v>
       </c>
       <c r="F14" s="10">
-        <f>SUM(F10:F13)</f>
-        <v>48</v>
+        <f>SUM(F12:F13)</f>
+        <v>42</v>
       </c>
       <c r="G14" s="10">
-        <f>SUM(G10:G13)</f>
-        <v>48</v>
+        <f>SUM(G12:G13)</f>
+        <v>42</v>
       </c>
       <c r="H14" s="10">
-        <f>SUM(H10:H13)</f>
-        <v>48</v>
+        <f>SUM(H12:H13)</f>
+        <v>42</v>
       </c>
       <c r="I14" s="10">
-        <f>SUM(I10:I13)</f>
-        <v>48</v>
+        <f>SUM(I12:I13)</f>
+        <v>42</v>
       </c>
       <c r="J14" s="10">
-        <f>SUM(J10:J13)</f>
-        <v>61</v>
+        <f>SUM(J12:J13)</f>
+        <v>52</v>
       </c>
       <c r="K14" s="10">
-        <f>SUM(K10:K13)</f>
-        <v>445</v>
+        <f>SUM(K12:K13)</f>
+        <v>388</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>Net Income</t>
+          <t>Gross Profit</t>
         </is>
       </c>
       <c r="B16" s="12">
         <f>B7-B14</f>
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="C16" s="12">
         <f>C7-C14</f>
-        <v>-48</v>
+        <v>-42</v>
       </c>
       <c r="D16" s="12">
         <f>D7-D14</f>
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="E16" s="12">
         <f>E7-E14</f>
-        <v>-48</v>
+        <v>-42</v>
       </c>
       <c r="F16" s="12">
         <f>F7-F14</f>
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="G16" s="12">
         <f>G7-G14</f>
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="H16" s="12">
         <f>H7-H14</f>
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="I16" s="12">
         <f>I7-I14</f>
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="J16" s="12">
         <f>J7-J14</f>
-        <v>-61</v>
+        <v>-52</v>
       </c>
       <c r="K16" s="12">
         <f>K7-K14</f>
+        <v>1097</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Operating Expenses</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="7" t="n"/>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+      <c r="H18" s="7" t="n"/>
+      <c r="I18" s="7" t="n"/>
+      <c r="J18" s="7" t="n"/>
+      <c r="K18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Bank Fees (GroupRB:Bank Fees)</t>
+        </is>
+      </c>
+      <c r="B19" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;B$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
+        <v>6</v>
+      </c>
+      <c r="C19" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;C$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
+        <v>6</v>
+      </c>
+      <c r="D19" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;D$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
+        <v>6</v>
+      </c>
+      <c r="E19" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;E$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
+        <v>6</v>
+      </c>
+      <c r="F19" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;F$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
+        <v>6</v>
+      </c>
+      <c r="G19" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;G$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
+        <v>6</v>
+      </c>
+      <c r="H19" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;H$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
+        <v>6</v>
+      </c>
+      <c r="I19" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;I$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
+        <v>6</v>
+      </c>
+      <c r="J19" s="9">
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;J$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
+        <v>9</v>
+      </c>
+      <c r="K19" s="9">
+        <f>SUM(B19:J19)</f>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Total Operating Expenses</t>
+        </is>
+      </c>
+      <c r="B20" s="10">
+        <f>SUM(B19:B19)</f>
+        <v>6</v>
+      </c>
+      <c r="C20" s="10">
+        <f>SUM(C19:C19)</f>
+        <v>6</v>
+      </c>
+      <c r="D20" s="10">
+        <f>SUM(D19:D19)</f>
+        <v>6</v>
+      </c>
+      <c r="E20" s="10">
+        <f>SUM(E19:E19)</f>
+        <v>6</v>
+      </c>
+      <c r="F20" s="10">
+        <f>SUM(F19:F19)</f>
+        <v>6</v>
+      </c>
+      <c r="G20" s="10">
+        <f>SUM(G19:G19)</f>
+        <v>6</v>
+      </c>
+      <c r="H20" s="10">
+        <f>SUM(H19:H19)</f>
+        <v>6</v>
+      </c>
+      <c r="I20" s="10">
+        <f>SUM(I19:I19)</f>
+        <v>6</v>
+      </c>
+      <c r="J20" s="10">
+        <f>SUM(J19:J19)</f>
+        <v>9</v>
+      </c>
+      <c r="K20" s="10">
+        <f>SUM(K19:K19)</f>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Net Income</t>
+        </is>
+      </c>
+      <c r="B22" s="13">
+        <f>B16-B20</f>
+        <v>150</v>
+      </c>
+      <c r="C22" s="13">
+        <f>C16-C20</f>
+        <v>-48</v>
+      </c>
+      <c r="D22" s="13">
+        <f>D16-D20</f>
+        <v>348</v>
+      </c>
+      <c r="E22" s="13">
+        <f>E16-E20</f>
+        <v>-48</v>
+      </c>
+      <c r="F22" s="13">
+        <f>F16-F20</f>
+        <v>150</v>
+      </c>
+      <c r="G22" s="13">
+        <f>G16-G20</f>
+        <v>150</v>
+      </c>
+      <c r="H22" s="13">
+        <f>H16-H20</f>
+        <v>150</v>
+      </c>
+      <c r="I22" s="13">
+        <f>I16-I20</f>
+        <v>249</v>
+      </c>
+      <c r="J22" s="13">
+        <f>J16-J20</f>
+        <v>-61</v>
+      </c>
+      <c r="K22" s="13">
+        <f>K16-K20</f>
         <v>1040</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="13" t="inlineStr">
-        <is>
-          <t>Notes / assumptions:</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
-        <is>
-          <t>- SEO &amp; Web Services revenue is pulled directly from the recorded Invoice rows in Revenue-source.xlsx (actual invoice dates, not evenly smoothed).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Feb and Apr show $0 because no invoice was recorded those months in the source file; Sep shows $0 because no Sep SEO &amp; Web Services invoice has been recorded yet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="14" t="inlineStr">
-        <is>
-          <t>- Hosting, Seobility, Ubersuggest and Billing Fee are GroupRB out-of-pocket costs to deliver Parts of Practice, entered per the schedule you gave:</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Hosting $10/mo and Billing Fee $3/mo — Andy Studer &amp; Gratitude Jan-Sep, Guidance Through Grief Sep only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Seobility $5/mo and Ubersuggest $6/mo — Andy Studer &amp; Gratitude only, Jan-Sep (not billed for Grief).</t>
-        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="14" t="inlineStr">
         <is>
-          <t>- "Billing Fee" is my label for the $3/mo charge described as "monthly billing charge" — rename in the Expense Detail sheet if you use a different name internally.</t>
+          <t>Notes / assumptions:</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="14" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>- SEO &amp; Web Services revenue is pulled directly from the recorded Invoice rows in Revenue-source.xlsx (actual invoice dates, not evenly smoothed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Feb and Apr show $0 because no invoice was recorded those months in the source file; Sep shows $0 because no Sep SEO &amp; Web Services invoice has been recorded yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>- Hosting and SEO Tools (Seobility + Ubersuggest) are classified as COGS: direct, per-client costs of delivering the SEO &amp; Web Services product.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>- Bank Fees ($3/mo QuickBooks Payments processing fee) is classified as an Operating Expense, not COGS, since it is a cost of collecting payment, not of delivering the service.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>- Schedule: Hosting $10/mo and Bank Fees $3/mo — Andy Studer &amp; Gratitude Jan-Sep, Guidance Through Grief Sep only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Seobility $5/mo and Ubersuggest $6/mo — Andy Studer &amp; Gratitude only, Jan-Sep (not billed for Grief).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>- The Expense Detail sheet has a "GL Account (Patriot)" column showing which account to code each transaction to when categorizing in Patriot.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>- Patriot true parent/child sub-accounts (e.g. GroupRB as parent of Hosting/SEO Tools/Bank Fees) require the Accounting Premium plan (up to 8 levels).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  On the Basic plan, naming an account "GroupRB:Hosting" creates a flat account with that literal name — it will not nest or roll up in reports.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>- All monthly charges are dated the 1st of the month per your instructions ("billed on the 1st").</t>
         </is>
@@ -1051,29 +1237,29 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="16" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="16" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="n">
+      <c r="A2" s="17" t="n">
         <v>46053</v>
       </c>
       <c r="B2" s="8" t="inlineStr">
@@ -1086,12 +1272,12 @@
           <t>SEO &amp; Web Services</t>
         </is>
       </c>
-      <c r="D2" s="17" t="n">
+      <c r="D2" s="18" t="n">
         <v>99</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="n">
+      <c r="A3" s="17" t="n">
         <v>46053</v>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1104,12 +1290,12 @@
           <t>SEO &amp; Web Services</t>
         </is>
       </c>
-      <c r="D3" s="17" t="n">
+      <c r="D3" s="18" t="n">
         <v>99</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="n">
+      <c r="A4" s="17" t="n">
         <v>46083</v>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -1122,12 +1308,12 @@
           <t>SEO &amp; Web Services</t>
         </is>
       </c>
-      <c r="D4" s="17" t="n">
+      <c r="D4" s="18" t="n">
         <v>99</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="n">
+      <c r="A5" s="17" t="n">
         <v>46083</v>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1140,12 +1326,12 @@
           <t>SEO &amp; Web Services</t>
         </is>
       </c>
-      <c r="D5" s="17" t="n">
+      <c r="D5" s="18" t="n">
         <v>99</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n">
+      <c r="A6" s="17" t="n">
         <v>46112</v>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -1158,12 +1344,12 @@
           <t>SEO &amp; Web Services</t>
         </is>
       </c>
-      <c r="D6" s="17" t="n">
+      <c r="D6" s="18" t="n">
         <v>99</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="n">
+      <c r="A7" s="17" t="n">
         <v>46112</v>
       </c>
       <c r="B7" s="8" t="inlineStr">
@@ -1176,12 +1362,12 @@
           <t>SEO &amp; Web Services</t>
         </is>
       </c>
-      <c r="D7" s="17" t="n">
+      <c r="D7" s="18" t="n">
         <v>99</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n">
+      <c r="A8" s="17" t="n">
         <v>46146</v>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -1194,12 +1380,12 @@
           <t>SEO &amp; Web Services</t>
         </is>
       </c>
-      <c r="D8" s="17" t="n">
+      <c r="D8" s="18" t="n">
         <v>99</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="n">
+      <c r="A9" s="17" t="n">
         <v>46146</v>
       </c>
       <c r="B9" s="8" t="inlineStr">
@@ -1212,12 +1398,12 @@
           <t>SEO &amp; Web Services</t>
         </is>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="D9" s="18" t="n">
         <v>99</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="n">
+      <c r="A10" s="17" t="n">
         <v>46181</v>
       </c>
       <c r="B10" s="8" t="inlineStr">
@@ -1230,12 +1416,12 @@
           <t>SEO &amp; Web Services</t>
         </is>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D10" s="18" t="n">
         <v>99</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="n">
+      <c r="A11" s="17" t="n">
         <v>46181</v>
       </c>
       <c r="B11" s="8" t="inlineStr">
@@ -1248,12 +1434,12 @@
           <t>SEO &amp; Web Services</t>
         </is>
       </c>
-      <c r="D11" s="17" t="n">
+      <c r="D11" s="18" t="n">
         <v>99</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="n">
+      <c r="A12" s="17" t="n">
         <v>46204</v>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -1266,12 +1452,12 @@
           <t>SEO &amp; Web Services</t>
         </is>
       </c>
-      <c r="D12" s="17" t="n">
+      <c r="D12" s="18" t="n">
         <v>99</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="n">
+      <c r="A13" s="17" t="n">
         <v>46204</v>
       </c>
       <c r="B13" s="8" t="inlineStr">
@@ -1284,12 +1470,12 @@
           <t>SEO &amp; Web Services</t>
         </is>
       </c>
-      <c r="D13" s="17" t="n">
+      <c r="D13" s="18" t="n">
         <v>99</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="n">
+      <c r="A14" s="17" t="n">
         <v>46239</v>
       </c>
       <c r="B14" s="8" t="inlineStr">
@@ -1302,12 +1488,12 @@
           <t>SEO &amp; Web Services</t>
         </is>
       </c>
-      <c r="D14" s="17" t="n">
+      <c r="D14" s="18" t="n">
         <v>99</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="n">
+      <c r="A15" s="17" t="n">
         <v>46239</v>
       </c>
       <c r="B15" s="8" t="inlineStr">
@@ -1320,12 +1506,12 @@
           <t>SEO &amp; Web Services</t>
         </is>
       </c>
-      <c r="D15" s="17" t="n">
+      <c r="D15" s="18" t="n">
         <v>99</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="n">
+      <c r="A16" s="17" t="n">
         <v>46239</v>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -1338,7 +1524,7 @@
           <t>SEO &amp; Web Services</t>
         </is>
       </c>
-      <c r="D16" s="17" t="n">
+      <c r="D16" s="18" t="n">
         <v>99</v>
       </c>
     </row>
@@ -1353,39 +1539,45 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D75"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>Customer</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="16" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="16" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
+      <c r="E1" s="16" t="inlineStr">
+        <is>
+          <t>GL Account (Patriot)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="n">
+      <c r="A2" s="19" t="n">
         <v>46023</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -1395,15 +1587,20 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D2" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D2" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E2" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="n">
+      <c r="A3" s="19" t="n">
         <v>46023</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -1413,15 +1610,20 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D3" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D3" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E3" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="n">
+      <c r="A4" s="19" t="n">
         <v>46023</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -1434,12 +1636,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D4" s="17" t="n">
+      <c r="D4" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="n">
+      <c r="A5" s="19" t="n">
         <v>46023</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -1452,12 +1659,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D5" s="17" t="n">
+      <c r="D5" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="n">
+      <c r="A6" s="19" t="n">
         <v>46023</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -1470,12 +1682,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D6" s="17" t="n">
+      <c r="D6" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="18" t="n">
+      <c r="A7" s="19" t="n">
         <v>46023</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -1488,12 +1705,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D7" s="17" t="n">
+      <c r="D7" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="n">
+      <c r="A8" s="19" t="n">
         <v>46023</v>
       </c>
       <c r="B8" t="inlineStr">
@@ -1506,12 +1728,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D8" s="17" t="n">
-        <v>6</v>
+      <c r="D8" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="n">
+      <c r="A9" s="19" t="n">
         <v>46023</v>
       </c>
       <c r="B9" t="inlineStr">
@@ -1524,12 +1751,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D9" s="17" t="n">
-        <v>6</v>
+      <c r="D9" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="n">
+      <c r="A10" s="19" t="n">
         <v>46054</v>
       </c>
       <c r="B10" t="inlineStr">
@@ -1539,15 +1771,20 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D10" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="n">
+      <c r="A11" s="19" t="n">
         <v>46054</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -1557,15 +1794,20 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D11" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E11" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="n">
+      <c r="A12" s="19" t="n">
         <v>46054</v>
       </c>
       <c r="B12" t="inlineStr">
@@ -1578,12 +1820,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D12" s="17" t="n">
+      <c r="D12" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="n">
+      <c r="A13" s="19" t="n">
         <v>46054</v>
       </c>
       <c r="B13" t="inlineStr">
@@ -1596,12 +1843,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D13" s="17" t="n">
+      <c r="D13" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E13" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="n">
+      <c r="A14" s="19" t="n">
         <v>46054</v>
       </c>
       <c r="B14" t="inlineStr">
@@ -1614,12 +1866,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D14" s="17" t="n">
+      <c r="D14" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E14" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="n">
+      <c r="A15" s="19" t="n">
         <v>46054</v>
       </c>
       <c r="B15" t="inlineStr">
@@ -1632,12 +1889,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D15" s="17" t="n">
+      <c r="D15" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E15" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="n">
+      <c r="A16" s="19" t="n">
         <v>46054</v>
       </c>
       <c r="B16" t="inlineStr">
@@ -1650,12 +1912,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D16" s="17" t="n">
-        <v>6</v>
+      <c r="D16" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="n">
+      <c r="A17" s="19" t="n">
         <v>46054</v>
       </c>
       <c r="B17" t="inlineStr">
@@ -1668,12 +1935,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D17" s="17" t="n">
-        <v>6</v>
+      <c r="D17" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="18" t="n">
+      <c r="A18" s="19" t="n">
         <v>46082</v>
       </c>
       <c r="B18" t="inlineStr">
@@ -1683,15 +1955,20 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D18" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="n">
+      <c r="A19" s="19" t="n">
         <v>46082</v>
       </c>
       <c r="B19" t="inlineStr">
@@ -1701,15 +1978,20 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D19" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E19" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="n">
+      <c r="A20" s="19" t="n">
         <v>46082</v>
       </c>
       <c r="B20" t="inlineStr">
@@ -1722,12 +2004,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D20" s="17" t="n">
+      <c r="D20" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E20" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="18" t="n">
+      <c r="A21" s="19" t="n">
         <v>46082</v>
       </c>
       <c r="B21" t="inlineStr">
@@ -1740,12 +2027,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D21" s="17" t="n">
+      <c r="D21" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E21" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="18" t="n">
+      <c r="A22" s="19" t="n">
         <v>46082</v>
       </c>
       <c r="B22" t="inlineStr">
@@ -1758,12 +2050,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D22" s="17" t="n">
+      <c r="D22" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="18" t="n">
+      <c r="A23" s="19" t="n">
         <v>46082</v>
       </c>
       <c r="B23" t="inlineStr">
@@ -1776,12 +2073,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D23" s="17" t="n">
+      <c r="D23" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E23" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="18" t="n">
+      <c r="A24" s="19" t="n">
         <v>46082</v>
       </c>
       <c r="B24" t="inlineStr">
@@ -1794,12 +2096,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D24" s="17" t="n">
-        <v>6</v>
+      <c r="D24" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="18" t="n">
+      <c r="A25" s="19" t="n">
         <v>46082</v>
       </c>
       <c r="B25" t="inlineStr">
@@ -1812,12 +2119,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D25" s="17" t="n">
-        <v>6</v>
+      <c r="D25" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E25" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="18" t="n">
+      <c r="A26" s="19" t="n">
         <v>46113</v>
       </c>
       <c r="B26" t="inlineStr">
@@ -1827,15 +2139,20 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D26" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="18" t="n">
+      <c r="A27" s="19" t="n">
         <v>46113</v>
       </c>
       <c r="B27" t="inlineStr">
@@ -1845,15 +2162,20 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D27" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E27" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="18" t="n">
+      <c r="A28" s="19" t="n">
         <v>46113</v>
       </c>
       <c r="B28" t="inlineStr">
@@ -1866,12 +2188,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D28" s="17" t="n">
+      <c r="D28" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E28" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="18" t="n">
+      <c r="A29" s="19" t="n">
         <v>46113</v>
       </c>
       <c r="B29" t="inlineStr">
@@ -1884,12 +2211,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D29" s="17" t="n">
+      <c r="D29" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E29" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="18" t="n">
+      <c r="A30" s="19" t="n">
         <v>46113</v>
       </c>
       <c r="B30" t="inlineStr">
@@ -1902,12 +2234,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D30" s="17" t="n">
+      <c r="D30" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E30" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="18" t="n">
+      <c r="A31" s="19" t="n">
         <v>46113</v>
       </c>
       <c r="B31" t="inlineStr">
@@ -1920,12 +2257,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D31" s="17" t="n">
+      <c r="D31" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E31" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="18" t="n">
+      <c r="A32" s="19" t="n">
         <v>46113</v>
       </c>
       <c r="B32" t="inlineStr">
@@ -1938,12 +2280,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D32" s="17" t="n">
-        <v>6</v>
+      <c r="D32" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E32" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="18" t="n">
+      <c r="A33" s="19" t="n">
         <v>46113</v>
       </c>
       <c r="B33" t="inlineStr">
@@ -1956,12 +2303,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D33" s="17" t="n">
-        <v>6</v>
+      <c r="D33" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E33" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="18" t="n">
+      <c r="A34" s="19" t="n">
         <v>46143</v>
       </c>
       <c r="B34" t="inlineStr">
@@ -1971,15 +2323,20 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D34" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D34" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E34" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="18" t="n">
+      <c r="A35" s="19" t="n">
         <v>46143</v>
       </c>
       <c r="B35" t="inlineStr">
@@ -1989,15 +2346,20 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D35" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D35" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E35" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="18" t="n">
+      <c r="A36" s="19" t="n">
         <v>46143</v>
       </c>
       <c r="B36" t="inlineStr">
@@ -2010,12 +2372,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D36" s="17" t="n">
+      <c r="D36" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E36" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="18" t="n">
+      <c r="A37" s="19" t="n">
         <v>46143</v>
       </c>
       <c r="B37" t="inlineStr">
@@ -2028,12 +2395,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D37" s="17" t="n">
+      <c r="D37" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E37" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="18" t="n">
+      <c r="A38" s="19" t="n">
         <v>46143</v>
       </c>
       <c r="B38" t="inlineStr">
@@ -2046,12 +2418,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D38" s="17" t="n">
+      <c r="D38" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E38" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="18" t="n">
+      <c r="A39" s="19" t="n">
         <v>46143</v>
       </c>
       <c r="B39" t="inlineStr">
@@ -2064,12 +2441,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D39" s="17" t="n">
+      <c r="D39" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E39" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="18" t="n">
+      <c r="A40" s="19" t="n">
         <v>46143</v>
       </c>
       <c r="B40" t="inlineStr">
@@ -2082,12 +2464,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D40" s="17" t="n">
-        <v>6</v>
+      <c r="D40" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E40" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="18" t="n">
+      <c r="A41" s="19" t="n">
         <v>46143</v>
       </c>
       <c r="B41" t="inlineStr">
@@ -2100,12 +2487,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D41" s="17" t="n">
-        <v>6</v>
+      <c r="D41" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E41" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="18" t="n">
+      <c r="A42" s="19" t="n">
         <v>46174</v>
       </c>
       <c r="B42" t="inlineStr">
@@ -2115,15 +2507,20 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D42" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D42" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E42" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="18" t="n">
+      <c r="A43" s="19" t="n">
         <v>46174</v>
       </c>
       <c r="B43" t="inlineStr">
@@ -2133,15 +2530,20 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D43" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D43" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E43" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="18" t="n">
+      <c r="A44" s="19" t="n">
         <v>46174</v>
       </c>
       <c r="B44" t="inlineStr">
@@ -2154,12 +2556,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D44" s="17" t="n">
+      <c r="D44" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E44" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="18" t="n">
+      <c r="A45" s="19" t="n">
         <v>46174</v>
       </c>
       <c r="B45" t="inlineStr">
@@ -2172,12 +2579,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D45" s="17" t="n">
+      <c r="D45" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E45" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="18" t="n">
+      <c r="A46" s="19" t="n">
         <v>46174</v>
       </c>
       <c r="B46" t="inlineStr">
@@ -2190,12 +2602,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D46" s="17" t="n">
+      <c r="D46" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E46" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="18" t="n">
+      <c r="A47" s="19" t="n">
         <v>46174</v>
       </c>
       <c r="B47" t="inlineStr">
@@ -2208,12 +2625,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D47" s="17" t="n">
+      <c r="D47" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E47" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="18" t="n">
+      <c r="A48" s="19" t="n">
         <v>46174</v>
       </c>
       <c r="B48" t="inlineStr">
@@ -2226,12 +2648,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D48" s="17" t="n">
-        <v>6</v>
+      <c r="D48" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E48" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="18" t="n">
+      <c r="A49" s="19" t="n">
         <v>46174</v>
       </c>
       <c r="B49" t="inlineStr">
@@ -2244,12 +2671,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D49" s="17" t="n">
-        <v>6</v>
+      <c r="D49" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E49" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="18" t="n">
+      <c r="A50" s="19" t="n">
         <v>46204</v>
       </c>
       <c r="B50" t="inlineStr">
@@ -2259,15 +2691,20 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D50" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D50" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E50" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="18" t="n">
+      <c r="A51" s="19" t="n">
         <v>46204</v>
       </c>
       <c r="B51" t="inlineStr">
@@ -2277,15 +2714,20 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D51" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D51" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E51" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="18" t="n">
+      <c r="A52" s="19" t="n">
         <v>46204</v>
       </c>
       <c r="B52" t="inlineStr">
@@ -2298,12 +2740,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D52" s="17" t="n">
+      <c r="D52" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E52" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="18" t="n">
+      <c r="A53" s="19" t="n">
         <v>46204</v>
       </c>
       <c r="B53" t="inlineStr">
@@ -2316,12 +2763,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D53" s="17" t="n">
+      <c r="D53" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E53" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="18" t="n">
+      <c r="A54" s="19" t="n">
         <v>46204</v>
       </c>
       <c r="B54" t="inlineStr">
@@ -2334,12 +2786,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D54" s="17" t="n">
+      <c r="D54" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E54" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="18" t="n">
+      <c r="A55" s="19" t="n">
         <v>46204</v>
       </c>
       <c r="B55" t="inlineStr">
@@ -2352,12 +2809,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D55" s="17" t="n">
+      <c r="D55" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E55" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="18" t="n">
+      <c r="A56" s="19" t="n">
         <v>46204</v>
       </c>
       <c r="B56" t="inlineStr">
@@ -2370,12 +2832,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D56" s="17" t="n">
-        <v>6</v>
+      <c r="D56" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E56" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="18" t="n">
+      <c r="A57" s="19" t="n">
         <v>46204</v>
       </c>
       <c r="B57" t="inlineStr">
@@ -2388,12 +2855,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D57" s="17" t="n">
-        <v>6</v>
+      <c r="D57" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E57" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="18" t="n">
+      <c r="A58" s="19" t="n">
         <v>46235</v>
       </c>
       <c r="B58" t="inlineStr">
@@ -2403,15 +2875,20 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D58" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D58" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E58" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="18" t="n">
+      <c r="A59" s="19" t="n">
         <v>46235</v>
       </c>
       <c r="B59" t="inlineStr">
@@ -2421,15 +2898,20 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D59" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D59" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E59" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="18" t="n">
+      <c r="A60" s="19" t="n">
         <v>46235</v>
       </c>
       <c r="B60" t="inlineStr">
@@ -2442,12 +2924,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D60" s="17" t="n">
+      <c r="D60" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E60" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="18" t="n">
+      <c r="A61" s="19" t="n">
         <v>46235</v>
       </c>
       <c r="B61" t="inlineStr">
@@ -2460,12 +2947,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D61" s="17" t="n">
+      <c r="D61" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E61" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="18" t="n">
+      <c r="A62" s="19" t="n">
         <v>46235</v>
       </c>
       <c r="B62" t="inlineStr">
@@ -2478,12 +2970,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D62" s="17" t="n">
+      <c r="D62" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E62" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="18" t="n">
+      <c r="A63" s="19" t="n">
         <v>46235</v>
       </c>
       <c r="B63" t="inlineStr">
@@ -2496,12 +2993,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D63" s="17" t="n">
+      <c r="D63" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E63" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="18" t="n">
+      <c r="A64" s="19" t="n">
         <v>46235</v>
       </c>
       <c r="B64" t="inlineStr">
@@ -2514,12 +3016,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D64" s="17" t="n">
-        <v>6</v>
+      <c r="D64" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E64" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="18" t="n">
+      <c r="A65" s="19" t="n">
         <v>46235</v>
       </c>
       <c r="B65" t="inlineStr">
@@ -2532,12 +3039,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D65" s="17" t="n">
-        <v>6</v>
+      <c r="D65" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E65" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="18" t="n">
+      <c r="A66" s="19" t="n">
         <v>46266</v>
       </c>
       <c r="B66" t="inlineStr">
@@ -2547,15 +3059,20 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D66" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D66" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E66" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="18" t="n">
+      <c r="A67" s="19" t="n">
         <v>46266</v>
       </c>
       <c r="B67" t="inlineStr">
@@ -2565,15 +3082,20 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D67" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D67" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E67" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" s="18" t="n">
+      <c r="A68" s="19" t="n">
         <v>46266</v>
       </c>
       <c r="B68" t="inlineStr">
@@ -2583,15 +3105,20 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Billing Fee</t>
-        </is>
-      </c>
-      <c r="D68" s="17" t="n">
+          <t>Bank Fees</t>
+        </is>
+      </c>
+      <c r="D68" s="18" t="n">
         <v>3</v>
       </c>
+      <c r="E68" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Bank Fees</t>
+        </is>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" s="18" t="n">
+      <c r="A69" s="19" t="n">
         <v>46266</v>
       </c>
       <c r="B69" t="inlineStr">
@@ -2604,12 +3131,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D69" s="17" t="n">
+      <c r="D69" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E69" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="18" t="n">
+      <c r="A70" s="19" t="n">
         <v>46266</v>
       </c>
       <c r="B70" t="inlineStr">
@@ -2622,12 +3154,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D70" s="17" t="n">
+      <c r="D70" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E70" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="18" t="n">
+      <c r="A71" s="19" t="n">
         <v>46266</v>
       </c>
       <c r="B71" t="inlineStr">
@@ -2640,12 +3177,17 @@
           <t>Hosting</t>
         </is>
       </c>
-      <c r="D71" s="17" t="n">
+      <c r="D71" s="18" t="n">
         <v>10</v>
       </c>
+      <c r="E71" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:Hosting</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="18" t="n">
+      <c r="A72" s="19" t="n">
         <v>46266</v>
       </c>
       <c r="B72" t="inlineStr">
@@ -2658,12 +3200,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D72" s="17" t="n">
+      <c r="D72" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E72" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" s="18" t="n">
+      <c r="A73" s="19" t="n">
         <v>46266</v>
       </c>
       <c r="B73" t="inlineStr">
@@ -2676,12 +3223,17 @@
           <t>Seobility</t>
         </is>
       </c>
-      <c r="D73" s="17" t="n">
+      <c r="D73" s="18" t="n">
         <v>5</v>
       </c>
+      <c r="E73" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="18" t="n">
+      <c r="A74" s="19" t="n">
         <v>46266</v>
       </c>
       <c r="B74" t="inlineStr">
@@ -2694,12 +3246,17 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D74" s="17" t="n">
-        <v>6</v>
+      <c r="D74" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E74" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="18" t="n">
+      <c r="A75" s="19" t="n">
         <v>46266</v>
       </c>
       <c r="B75" t="inlineStr">
@@ -2712,8 +3269,13 @@
           <t>Ubersuggest</t>
         </is>
       </c>
-      <c r="D75" s="17" t="n">
-        <v>6</v>
+      <c r="D75" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E75" s="20" t="inlineStr">
+        <is>
+          <t>GroupRB:SEO Tools</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Match GL account names to the chart of accounts actually set up in Patriot
Rename accounts to Hosting Fees and SEO Tools (subaccounts of Cost of
Goods Sold) and reuse the existing Bank Processing Fees expense
account instead of the placeholder GroupRB:* names. Applies to the
P&L, Expense Detail's GL Account column, and the Patriot import
descriptions.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EWHJ4JSrXozykE2fwAhg1g
</commit_message>
<xml_diff>
--- a/Practice Budget Expenses Revenue Conversion/2026 P&L by Month.xlsx
+++ b/Practice Budget Expenses Revenue Conversion/2026 P&L by Month.xlsx
@@ -796,7 +796,7 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>SEO Tools (GroupRB:SEO Tools)</t>
+          <t>SEO Tools</t>
         </is>
       </c>
       <c r="B12" s="9">
@@ -843,43 +843,43 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Hosting (GroupRB:Hosting)</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="B13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;B$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting Fees",'Expense Detail'!$A:$A,"&gt;="&amp;B$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
         <v>20</v>
       </c>
       <c r="C13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;C$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting Fees",'Expense Detail'!$A:$A,"&gt;="&amp;C$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
         <v>20</v>
       </c>
       <c r="D13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;D$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting Fees",'Expense Detail'!$A:$A,"&gt;="&amp;D$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
         <v>20</v>
       </c>
       <c r="E13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;E$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting Fees",'Expense Detail'!$A:$A,"&gt;="&amp;E$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
         <v>20</v>
       </c>
       <c r="F13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;F$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting Fees",'Expense Detail'!$A:$A,"&gt;="&amp;F$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
         <v>20</v>
       </c>
       <c r="G13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;G$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting Fees",'Expense Detail'!$A:$A,"&gt;="&amp;G$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
         <v>20</v>
       </c>
       <c r="H13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;H$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting Fees",'Expense Detail'!$A:$A,"&gt;="&amp;H$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
         <v>20</v>
       </c>
       <c r="I13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;I$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting Fees",'Expense Detail'!$A:$A,"&gt;="&amp;I$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
         <v>20</v>
       </c>
       <c r="J13" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting",'Expense Detail'!$A:$A,"&gt;="&amp;J$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Hosting Fees",'Expense Detail'!$A:$A,"&gt;="&amp;J$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
         <v>30</v>
       </c>
       <c r="K13" s="9">
@@ -1001,43 +1001,43 @@
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Bank Fees (GroupRB:Bank Fees)</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="B19" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;B$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Processing Fees",'Expense Detail'!$A:$A,"&gt;="&amp;B$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(B$4,1))</f>
         <v>6</v>
       </c>
       <c r="C19" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;C$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Processing Fees",'Expense Detail'!$A:$A,"&gt;="&amp;C$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(C$4,1))</f>
         <v>6</v>
       </c>
       <c r="D19" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;D$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Processing Fees",'Expense Detail'!$A:$A,"&gt;="&amp;D$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(D$4,1))</f>
         <v>6</v>
       </c>
       <c r="E19" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;E$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Processing Fees",'Expense Detail'!$A:$A,"&gt;="&amp;E$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(E$4,1))</f>
         <v>6</v>
       </c>
       <c r="F19" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;F$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Processing Fees",'Expense Detail'!$A:$A,"&gt;="&amp;F$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(F$4,1))</f>
         <v>6</v>
       </c>
       <c r="G19" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;G$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Processing Fees",'Expense Detail'!$A:$A,"&gt;="&amp;G$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(G$4,1))</f>
         <v>6</v>
       </c>
       <c r="H19" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;H$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Processing Fees",'Expense Detail'!$A:$A,"&gt;="&amp;H$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(H$4,1))</f>
         <v>6</v>
       </c>
       <c r="I19" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;I$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Processing Fees",'Expense Detail'!$A:$A,"&gt;="&amp;I$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(I$4,1))</f>
         <v>6</v>
       </c>
       <c r="J19" s="9">
-        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Fees",'Expense Detail'!$A:$A,"&gt;="&amp;J$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
+        <f>SUMIFS('Expense Detail'!$D:$D,'Expense Detail'!$C:$C,"Bank Processing Fees",'Expense Detail'!$A:$A,"&gt;="&amp;J$4,'Expense Detail'!$A:$A,"&lt;"&amp;EDATE(J$4,1))</f>
         <v>9</v>
       </c>
       <c r="K19" s="9">
@@ -1163,49 +1163,49 @@
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>- Hosting and SEO Tools (Seobility + Ubersuggest) are classified as COGS: direct, per-client costs of delivering the SEO &amp; Web Services product.</t>
+          <t>- Hosting Fees and SEO Tools (Seobility + Ubersuggest) are classified as COGS: direct, per-client costs of delivering the SEO &amp; Web Services product.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>- Bank Fees ($3/mo QuickBooks Payments processing fee) is classified as an Operating Expense, not COGS, since it is a cost of collecting payment, not of delivering the service.</t>
+          <t xml:space="preserve">  In Patriot they are subaccounts of Cost of Goods Sold, matching the chart of accounts you set up (Cost of Goods Sold &gt; SEO Tools, Hosting Fees).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="15" t="inlineStr">
         <is>
-          <t>- Schedule: Hosting $10/mo and Bank Fees $3/mo — Andy Studer &amp; Gratitude Jan-Sep, Guidance Through Grief Sep only.</t>
+          <t>- Bank Processing Fees ($3/mo QuickBooks Payments processing fee) is classified as an Operating Expense, not COGS, since it is a cost of collecting</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Seobility $5/mo and Ubersuggest $6/mo — Andy Studer &amp; Gratitude only, Jan-Sep (not billed for Grief).</t>
+          <t xml:space="preserve">  payment, not of delivering the service. Uses your existing Bank Processing Fees account rather than a new one.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t>- The Expense Detail sheet has a "GL Account (Patriot)" column showing which account to code each transaction to when categorizing in Patriot.</t>
+          <t>- Schedule: Hosting Fees $10/mo and Bank Processing Fees $3/mo — Andy Studer &amp; Gratitude Jan-Sep, Guidance Through Grief Sep only.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>- Patriot true parent/child sub-accounts (e.g. GroupRB as parent of Hosting/SEO Tools/Bank Fees) require the Accounting Premium plan (up to 8 levels).</t>
+          <t xml:space="preserve">  Seobility $5/mo and Ubersuggest $6/mo — Andy Studer &amp; Gratitude only, Jan-Sep (not billed for Grief).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">  On the Basic plan, naming an account "GroupRB:Hosting" creates a flat account with that literal name — it will not nest or roll up in reports.</t>
+          <t>- The Expense Detail sheet has a "GL Account (Patriot)" column showing which account to code each transaction to when categorizing in Patriot.</t>
         </is>
       </c>
     </row>
@@ -1587,7 +1587,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D2" s="18" t="n">
@@ -1595,7 +1595,7 @@
       </c>
       <c r="E2" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D3" s="18" t="n">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="E3" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D4" s="18" t="n">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="E4" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D5" s="18" t="n">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="E5" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1710,7 @@
       </c>
       <c r="E7" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="E9" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D10" s="18" t="n">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="E10" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D11" s="18" t="n">
@@ -1802,7 +1802,7 @@
       </c>
       <c r="E11" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1817,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D12" s="18" t="n">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="E12" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D13" s="18" t="n">
@@ -1848,7 +1848,7 @@
       </c>
       <c r="E13" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="E14" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1894,7 @@
       </c>
       <c r="E15" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1917,7 @@
       </c>
       <c r="E16" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -1940,7 +1940,7 @@
       </c>
       <c r="E17" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -1955,7 +1955,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D18" s="18" t="n">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="E18" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D19" s="18" t="n">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="E19" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D20" s="18" t="n">
@@ -2009,7 +2009,7 @@
       </c>
       <c r="E20" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2024,7 +2024,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D21" s="18" t="n">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="E21" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2055,7 +2055,7 @@
       </c>
       <c r="E22" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2078,7 +2078,7 @@
       </c>
       <c r="E23" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="E24" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2124,7 +2124,7 @@
       </c>
       <c r="E25" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2139,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D26" s="18" t="n">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="E26" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -2162,7 +2162,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D27" s="18" t="n">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="E27" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -2185,7 +2185,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D28" s="18" t="n">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="E28" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D29" s="18" t="n">
@@ -2216,7 +2216,7 @@
       </c>
       <c r="E29" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2239,7 +2239,7 @@
       </c>
       <c r="E30" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="E31" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="E32" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2308,7 +2308,7 @@
       </c>
       <c r="E33" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D34" s="18" t="n">
@@ -2331,7 +2331,7 @@
       </c>
       <c r="E34" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -2346,7 +2346,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D35" s="18" t="n">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="E35" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -2369,7 +2369,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D36" s="18" t="n">
@@ -2377,7 +2377,7 @@
       </c>
       <c r="E36" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D37" s="18" t="n">
@@ -2400,7 +2400,7 @@
       </c>
       <c r="E37" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2423,7 @@
       </c>
       <c r="E38" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2446,7 +2446,7 @@
       </c>
       <c r="E39" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="E40" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="E41" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2507,7 +2507,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D42" s="18" t="n">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="E42" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -2530,7 +2530,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D43" s="18" t="n">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="E43" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -2553,7 +2553,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D44" s="18" t="n">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="E44" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D45" s="18" t="n">
@@ -2584,7 +2584,7 @@
       </c>
       <c r="E45" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="E46" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2630,7 +2630,7 @@
       </c>
       <c r="E47" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2653,7 +2653,7 @@
       </c>
       <c r="E48" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="E49" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2691,7 +2691,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D50" s="18" t="n">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="E50" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D51" s="18" t="n">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="E51" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -2737,7 +2737,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D52" s="18" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="E52" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2760,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D53" s="18" t="n">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="E53" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2791,7 +2791,7 @@
       </c>
       <c r="E54" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2814,7 +2814,7 @@
       </c>
       <c r="E55" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2837,7 +2837,7 @@
       </c>
       <c r="E56" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2860,7 +2860,7 @@
       </c>
       <c r="E57" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D58" s="18" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="E58" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2898,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D59" s="18" t="n">
@@ -2906,7 +2906,7 @@
       </c>
       <c r="E59" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -2921,7 +2921,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D60" s="18" t="n">
@@ -2929,7 +2929,7 @@
       </c>
       <c r="E60" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D61" s="18" t="n">
@@ -2952,7 +2952,7 @@
       </c>
       <c r="E61" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2975,7 +2975,7 @@
       </c>
       <c r="E62" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -2998,7 +2998,7 @@
       </c>
       <c r="E63" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="E64" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -3044,7 +3044,7 @@
       </c>
       <c r="E65" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -3059,7 +3059,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D66" s="18" t="n">
@@ -3067,7 +3067,7 @@
       </c>
       <c r="E66" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -3082,7 +3082,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D67" s="18" t="n">
@@ -3090,7 +3090,7 @@
       </c>
       <c r="E67" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -3105,7 +3105,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
       <c r="D68" s="18" t="n">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="E68" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Bank Fees</t>
+          <t>Bank Processing Fees</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D69" s="18" t="n">
@@ -3136,7 +3136,7 @@
       </c>
       <c r="E69" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D70" s="18" t="n">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="E70" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -3174,7 +3174,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Hosting</t>
+          <t>Hosting Fees</t>
         </is>
       </c>
       <c r="D71" s="18" t="n">
@@ -3182,7 +3182,7 @@
       </c>
       <c r="E71" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:Hosting</t>
+          <t>Hosting Fees (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -3205,7 +3205,7 @@
       </c>
       <c r="E72" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3228,7 @@
       </c>
       <c r="E73" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="E74" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>
@@ -3274,7 +3274,7 @@
       </c>
       <c r="E75" s="20" t="inlineStr">
         <is>
-          <t>GroupRB:SEO Tools</t>
+          <t>SEO Tools (sub of Cost of Goods Sold)</t>
         </is>
       </c>
     </row>

</xml_diff>